<commit_message>
Proposal v2: inflation-based pricing with three options spanning 1403-based to 1404-based tariffs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FsX1FBErcEYRjqCBnDJRWY
</commit_message>
<xml_diff>
--- a/tariff_inflation_comparison.xlsx
+++ b/tariff_inflation_comparison.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="66">
   <si>
     <t xml:space="preserve">ماه</t>
   </si>
@@ -1623,6 +1623,49 @@
       </rPr>
       <t xml:space="preserve">تورم تا شهریور ۱۴۰۵</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">گزینه ۲ پروپوزال </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="FreeSans"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">میانگین گزینه ۱ و ۳</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">میانگین نرخ‌ها</t>
   </si>
   <si>
     <r>
@@ -2902,7 +2945,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -3135,19 +3178,56 @@
         <v>1.71101888883947</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
         <v>61</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>2.455</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>93.45</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>155.09</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>25302.9</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>313.3</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>13499.2</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>44997.3</v>
+      </c>
+      <c r="J7" s="8" t="n">
+        <f aca="false">I7/1000</f>
+        <v>44.9973</v>
+      </c>
+      <c r="K7" s="8" t="n">
+        <f aca="false">I7/$I$5</f>
+        <v>1.53947976146896</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>